<commit_message>
test(qa): distinguish upstream blocking from code faults in the patent test
TC-I-011 asserted `all(e.kind == "patent" for e in ev)`, which is vacuously
true on an empty list — so it passed while the fetcher was returning nothing
at all. Google now serves a 503 anti-bot page for the scraped
patents.google.com/xhr/query endpoint, blocking this host.

The test now probes upstream when the result is empty and reports BLOCKED with
the cause, rather than a silent pass. Patent evidence is unavailable until the
block clears or the fetcher moves to a supported API.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/REFlect_AI_Test_Report.xlsx
+++ b/qa/REFlect_AI_Test_Report.xlsx
@@ -69,7 +69,7 @@
       <color rgb="009C6500"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +139,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-07 13:38</t>
+          <t>Generated 2026-09-07 13:50</t>
         </is>
       </c>
     </row>
@@ -574,7 +582,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -594,7 +602,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -615,7 +623,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>97.8%</t>
         </is>
       </c>
     </row>
@@ -677,7 +685,7 @@
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -763,7 +771,7 @@
         <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -1682,7 +1690,7 @@
         </is>
       </c>
       <c r="L13" s="7" t="n">
-        <v>0.077</v>
+        <v>0.059</v>
       </c>
       <c r="M13" s="7" t="inlineStr"/>
       <c r="N13" s="7" t="inlineStr">
@@ -1748,7 +1756,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.136</v>
+        <v>0.138</v>
       </c>
       <c r="M14" s="7" t="inlineStr"/>
       <c r="N14" s="7" t="inlineStr">
@@ -1814,7 +1822,7 @@
         </is>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.013</v>
+        <v>0.023</v>
       </c>
       <c r="M15" s="7" t="inlineStr"/>
       <c r="N15" s="7" t="inlineStr">
@@ -1880,7 +1888,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.013</v>
+        <v>0.025</v>
       </c>
       <c r="M16" s="7" t="inlineStr"/>
       <c r="N16" s="7" t="inlineStr">
@@ -1946,7 +1954,7 @@
         </is>
       </c>
       <c r="L17" s="7" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="M17" s="7" t="inlineStr"/>
       <c r="N17" s="7" t="inlineStr">
@@ -2012,7 +2020,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="7" t="inlineStr">
@@ -2279,7 +2287,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.064</v>
+        <v>0.058</v>
       </c>
       <c r="M22" s="7" t="inlineStr"/>
       <c r="N22" s="7" t="inlineStr">
@@ -2336,18 +2344,22 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>0 items, kinds=[]</t>
-        </is>
-      </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>0 items; upstream probe HTTP 503</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.496</v>
-      </c>
-      <c r="M23" s="7" t="inlineStr"/>
+        <v>0.911</v>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>('M:\\REFlect_AI\\Impact_Lab\\qa\\test_integration.py', 149, 'Skipped: Google Patents is blocking this host (HTTP 503 anti-bot page). Scraped XHR endpoint, not a supported API - patent evidence will be empty.')</t>
+        </is>
+      </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
           <t>qa/test_integration.py::test_patent_fetcher</t>
@@ -2412,7 +2424,7 @@
         </is>
       </c>
       <c r="L24" s="7" t="n">
-        <v>0.819</v>
+        <v>1.17</v>
       </c>
       <c r="M24" s="7" t="inlineStr"/>
       <c r="N24" s="7" t="inlineStr">
@@ -2478,7 +2490,7 @@
         </is>
       </c>
       <c r="L25" s="7" t="n">
-        <v>0.023</v>
+        <v>0.013</v>
       </c>
       <c r="M25" s="7" t="inlineStr"/>
       <c r="N25" s="7" t="inlineStr">
@@ -2544,7 +2556,7 @@
         </is>
       </c>
       <c r="L26" s="7" t="n">
-        <v>0.022</v>
+        <v>0.026</v>
       </c>
       <c r="M26" s="7" t="inlineStr"/>
       <c r="N26" s="7" t="inlineStr">
@@ -2610,7 +2622,7 @@
         </is>
       </c>
       <c r="L27" s="7" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="M27" s="7" t="inlineStr"/>
       <c r="N27" s="7" t="inlineStr">
@@ -2676,7 +2688,7 @@
         </is>
       </c>
       <c r="L28" s="7" t="n">
-        <v>0.023</v>
+        <v>0.025</v>
       </c>
       <c r="M28" s="7" t="inlineStr"/>
       <c r="N28" s="7" t="inlineStr">
@@ -2742,7 +2754,7 @@
         </is>
       </c>
       <c r="L29" s="7" t="n">
-        <v>0.012</v>
+        <v>0.023</v>
       </c>
       <c r="M29" s="7" t="inlineStr"/>
       <c r="N29" s="7" t="inlineStr">
@@ -2809,7 +2821,7 @@
         </is>
       </c>
       <c r="L30" s="7" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
       <c r="M30" s="7" t="inlineStr"/>
       <c r="N30" s="7" t="inlineStr">
@@ -2876,7 +2888,7 @@
         </is>
       </c>
       <c r="L31" s="7" t="n">
-        <v>0.028</v>
+        <v>0.026</v>
       </c>
       <c r="M31" s="7" t="inlineStr"/>
       <c r="N31" s="7" t="inlineStr">
@@ -2943,7 +2955,7 @@
         </is>
       </c>
       <c r="L32" s="7" t="n">
-        <v>0.055</v>
+        <v>0.054</v>
       </c>
       <c r="M32" s="7" t="inlineStr"/>
       <c r="N32" s="7" t="inlineStr">
@@ -3010,7 +3022,7 @@
         </is>
       </c>
       <c r="L33" s="7" t="n">
-        <v>0.122</v>
+        <v>0.112</v>
       </c>
       <c r="M33" s="7" t="inlineStr"/>
       <c r="N33" s="7" t="inlineStr">
@@ -3211,7 +3223,7 @@
         </is>
       </c>
       <c r="L36" s="7" t="n">
-        <v>0.144</v>
+        <v>0.628</v>
       </c>
       <c r="M36" s="7" t="inlineStr"/>
       <c r="N36" s="7" t="inlineStr">
@@ -3278,7 +3290,7 @@
         </is>
       </c>
       <c r="L37" s="7" t="n">
-        <v>0.507</v>
+        <v>0.508</v>
       </c>
       <c r="M37" s="7" t="inlineStr"/>
       <c r="N37" s="7" t="inlineStr">
@@ -3345,7 +3357,7 @@
         </is>
       </c>
       <c r="L38" s="7" t="n">
-        <v>0.106</v>
+        <v>0.1</v>
       </c>
       <c r="M38" s="7" t="inlineStr"/>
       <c r="N38" s="7" t="inlineStr">
@@ -3403,7 +3415,7 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>mean=15.9 ms, max=22.5 ms over 5 calls</t>
+          <t>mean=13.8 ms, max=22.9 ms over 5 calls</t>
         </is>
       </c>
       <c r="K39" s="9" t="inlineStr">
@@ -3412,7 +3424,7 @@
         </is>
       </c>
       <c r="L39" s="7" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M39" s="7" t="inlineStr"/>
       <c r="N39" s="7" t="inlineStr">
@@ -3469,7 +3481,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>0.08 s to loaded</t>
+          <t>0.13 s to loaded</t>
         </is>
       </c>
       <c r="K40" s="9" t="inlineStr">
@@ -3478,7 +3490,7 @@
         </is>
       </c>
       <c r="L40" s="7" t="n">
-        <v>0.08</v>
+        <v>0.128</v>
       </c>
       <c r="M40" s="7" t="inlineStr"/>
       <c r="N40" s="7" t="inlineStr">
@@ -3536,7 +3548,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>0.0001 ms per cache hit</t>
+          <t>0.0002 ms per cache hit</t>
         </is>
       </c>
       <c r="K41" s="9" t="inlineStr">
@@ -3545,7 +3557,7 @@
         </is>
       </c>
       <c r="L41" s="7" t="n">
-        <v>0.093</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="M41" s="7" t="inlineStr"/>
       <c r="N41" s="7" t="inlineStr">
@@ -3603,7 +3615,7 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>20 concurrent in 0.08s, non-200=0</t>
+          <t>20 concurrent in 0.09s, non-200=0</t>
         </is>
       </c>
       <c r="K42" s="9" t="inlineStr">
@@ -3612,7 +3624,7 @@
         </is>
       </c>
       <c r="L42" s="7" t="n">
-        <v>0.079</v>
+        <v>0.094</v>
       </c>
       <c r="M42" s="7" t="inlineStr"/>
       <c r="N42" s="7" t="inlineStr">
@@ -3678,7 +3690,7 @@
         </is>
       </c>
       <c r="L43" s="7" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="M43" s="7" t="inlineStr"/>
       <c r="N43" s="7" t="inlineStr">
@@ -3803,7 +3815,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>scanned 20822 bytes across 3 endpoints; leaks=none</t>
+          <t>scanned 20837 bytes across 3 endpoints; leaks=none</t>
         </is>
       </c>
       <c r="K45" s="9" t="inlineStr">
@@ -3812,7 +3824,7 @@
         </is>
       </c>
       <c r="L45" s="7" t="n">
-        <v>0.057</v>
+        <v>0.064</v>
       </c>
       <c r="M45" s="7" t="inlineStr"/>
       <c r="N45" s="7" t="inlineStr">
@@ -3879,7 +3891,7 @@
         </is>
       </c>
       <c r="L46" s="7" t="n">
-        <v>0.904</v>
+        <v>0.905</v>
       </c>
       <c r="M46" s="7" t="inlineStr"/>
       <c r="N46" s="7" t="inlineStr">
@@ -3945,7 +3957,7 @@
         </is>
       </c>
       <c r="L47" s="7" t="n">
-        <v>0.031</v>
+        <v>0.03</v>
       </c>
       <c r="M47" s="7" t="inlineStr"/>
       <c r="N47" s="7" t="inlineStr">
@@ -4030,47 +4042,48 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DEF-001</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TC-I-011</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Fetchers</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>No defects open. All executed cases passed.</t>
+          <t>Patent fetcher executes without error</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Returns a list without raising; any items carry kind='patent'.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0 items; upstream probe HTTP 503
+('M:\\REFlect_AI\\Impact_Lab\\qa\\test_integration.py', 149, 'Skipped: Google Patents is blocking this host (HTTP 503 anti-bot page). Scraped XHR endpoint, not a supported API - patent evidence will be empty.')</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>